<commit_message>
recent course changes: 2026-10-24 22:11:33
</commit_message>
<xml_diff>
--- a/Курс 3/Проектирование БД/Курисовая/Книга1.xlsx
+++ b/Курс 3/Проектирование БД/Курисовая/Книга1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/olesteep/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OleSTEEP\Documents\Курисовая\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F0ABA20-BBAA-EB4E-9ABF-1553A657E65E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FCAEB80-577B-470E-AA03-8D5A2CB77EC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="25220" windowHeight="21680" xr2:uid="{E8ABD04A-C744-9645-AB57-F5C229AE1FFB}"/>
+    <workbookView xWindow="25695" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{E8ABD04A-C744-9645-AB57-F5C229AE1FFB}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="463" uniqueCount="207">
   <si>
     <t>Дата сделки</t>
   </si>
@@ -437,9 +437,6 @@
     <t>Монолитные</t>
   </si>
   <si>
-    <t>год постройки дома</t>
-  </si>
-  <si>
     <t>Кринкин Олег Алексеевич</t>
   </si>
   <si>
@@ -594,13 +591,79 @@
   </si>
   <si>
     <t>22.04.2026</t>
+  </si>
+  <si>
+    <t>12.03.1982</t>
+  </si>
+  <si>
+    <t>01.04.2012</t>
+  </si>
+  <si>
+    <t>23.12.1964</t>
+  </si>
+  <si>
+    <t>11.08.1959</t>
+  </si>
+  <si>
+    <t>30.07.1981</t>
+  </si>
+  <si>
+    <t>15.05.1967</t>
+  </si>
+  <si>
+    <t>10.09.2015</t>
+  </si>
+  <si>
+    <t>18.03.1970</t>
+  </si>
+  <si>
+    <t>21.06.2007</t>
+  </si>
+  <si>
+    <t>дата постройки дома</t>
+  </si>
+  <si>
+    <t>12.08.1978</t>
+  </si>
+  <si>
+    <t>Дата рождения владельца</t>
+  </si>
+  <si>
+    <t>10.09.2005</t>
+  </si>
+  <si>
+    <t>12.03.1976</t>
+  </si>
+  <si>
+    <t>12.07.1994</t>
+  </si>
+  <si>
+    <t>20.12.2000</t>
+  </si>
+  <si>
+    <t>11.08.1978</t>
+  </si>
+  <si>
+    <t>30.07.1974</t>
+  </si>
+  <si>
+    <t>15.05.1982</t>
+  </si>
+  <si>
+    <t>14.11.1994</t>
+  </si>
+  <si>
+    <t>22.02.1953</t>
+  </si>
+  <si>
+    <t>28.05.1992</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -639,6 +702,13 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -648,7 +718,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -682,11 +752,50 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -695,18 +804,23 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -1041,42 +1155,42 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66A0031D-02F4-BF44-AE14-59C0D6C26D55}">
-  <dimension ref="A1:BM23"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:BN17"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="11.6640625" customWidth="1"/>
+    <col min="1" max="1" width="11.625" customWidth="1"/>
     <col min="5" max="5" width="13" customWidth="1"/>
-    <col min="6" max="6" width="12.1640625" customWidth="1"/>
+    <col min="6" max="6" width="12.125" customWidth="1"/>
     <col min="8" max="8" width="15.5" customWidth="1"/>
     <col min="9" max="9" width="12.5" customWidth="1"/>
-    <col min="10" max="10" width="12.83203125" customWidth="1"/>
-    <col min="13" max="13" width="12.1640625" customWidth="1"/>
-    <col min="15" max="15" width="28.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.875" customWidth="1"/>
+    <col min="13" max="13" width="12.125" customWidth="1"/>
+    <col min="15" max="15" width="28.625" bestFit="1" customWidth="1"/>
     <col min="16" max="17" width="11" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="15.6640625" customWidth="1"/>
-    <col min="20" max="20" width="28.5" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="22.33203125" customWidth="1"/>
+    <col min="18" max="18" width="12.625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="15.625" customWidth="1"/>
+    <col min="20" max="20" width="14.75" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="22.375" customWidth="1"/>
     <col min="26" max="26" width="15" customWidth="1"/>
-    <col min="27" max="27" width="14.33203125" customWidth="1"/>
+    <col min="27" max="27" width="14.375" customWidth="1"/>
     <col min="28" max="28" width="25.5" bestFit="1" customWidth="1"/>
     <col min="31" max="31" width="11" bestFit="1" customWidth="1"/>
     <col min="35" max="35" width="14" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="14.6640625" customWidth="1"/>
-    <col min="38" max="38" width="21.1640625" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="14.625" customWidth="1"/>
+    <col min="38" max="38" width="21.125" bestFit="1" customWidth="1"/>
     <col min="44" max="44" width="13" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="13.83203125" customWidth="1"/>
-    <col min="47" max="47" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="23.83203125" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="13.1640625" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="21.6640625" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.83203125" customWidth="1"/>
-    <col min="61" max="61" width="17.1640625" customWidth="1"/>
-    <col min="62" max="62" width="12.1640625" customWidth="1"/>
-    <col min="63" max="63" width="13.1640625" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="13.875" customWidth="1"/>
+    <col min="47" max="47" width="12.875" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="23.875" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="13.125" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="21.625" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.875" customWidth="1"/>
+    <col min="61" max="61" width="17.125" customWidth="1"/>
+    <col min="62" max="62" width="12.125" customWidth="1"/>
+    <col min="63" max="63" width="13.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:65" ht="68" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:66" ht="63">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1131,154 +1245,157 @@
       <c r="R1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" s="14" t="s">
+        <v>196</v>
+      </c>
+      <c r="T1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="1" t="s">
+      <c r="AG1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" s="1" t="s">
+      <c r="AH1" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="AH1" s="1" t="s">
+      <c r="AI1" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="AI1" s="1" t="s">
+      <c r="AJ1" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="AJ1" s="1" t="s">
+      <c r="AK1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="AK1" s="1" t="s">
+      <c r="AL1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="AL1" s="1" t="s">
+      <c r="AM1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="AM1" s="1" t="s">
+      <c r="AN1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="AN1" s="1" t="s">
+      <c r="AO1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AO1" s="1" t="s">
+      <c r="AP1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="AP1" s="1" t="s">
+      <c r="AQ1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AQ1" s="1" t="s">
+      <c r="AR1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="AR1" s="1" t="s">
+      <c r="AS1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="AS1" s="1" t="s">
+      <c r="AT1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="AT1" s="1" t="s">
+      <c r="AU1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="AU1" s="1" t="s">
+      <c r="AV1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="AV1" s="1" t="s">
+      <c r="AW1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="AW1" s="1" t="s">
+      <c r="AX1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="AX1" s="1" t="s">
+      <c r="AY1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="AY1" s="1" t="s">
+      <c r="AZ1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="AZ1" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="BA1" s="1" t="s">
+      <c r="BA1" s="12" t="s">
+        <v>194</v>
+      </c>
+      <c r="BB1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="BB1" s="1" t="s">
+      <c r="BC1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="BC1" s="1" t="s">
+      <c r="BD1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="BD1" s="1" t="s">
+      <c r="BE1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="BE1" s="1" t="s">
+      <c r="BF1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="BF1" s="1" t="s">
+      <c r="BG1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="BG1" s="1" t="s">
+      <c r="BH1" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="BH1" s="1" t="s">
+      <c r="BI1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="BI1" s="1" t="s">
+      <c r="BJ1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="BJ1" s="1" t="s">
+      <c r="BK1" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="BK1" s="1" t="s">
+      <c r="BL1" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="BL1" s="1" t="s">
+      <c r="BM1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="BM1" s="1" t="s">
+      <c r="BN1" s="1" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="2" spans="1:65" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:66">
       <c r="A2" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C2" s="2">
         <v>19000</v>
@@ -1290,7 +1407,7 @@
         <v>25000</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>69</v>
@@ -1317,7 +1434,7 @@
         <v>40</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="P2" s="2">
         <v>1919</v>
@@ -1325,152 +1442,155 @@
       <c r="Q2" s="2">
         <v>472394</v>
       </c>
-      <c r="R2" s="7">
+      <c r="R2" s="5">
         <v>26491261361</v>
       </c>
-      <c r="S2" s="7">
+      <c r="S2" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="T2" s="5">
         <v>79232353057</v>
       </c>
-      <c r="T2" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="U2" s="9" t="s">
+      <c r="U2" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="V2" s="7" t="s">
         <v>62</v>
-      </c>
-      <c r="V2" s="2" t="s">
-        <v>165</v>
       </c>
       <c r="W2" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="X2" s="5">
+      <c r="X2" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="Y2" s="5">
         <v>1925</v>
       </c>
-      <c r="Y2" s="4">
+      <c r="Z2" s="4">
         <v>570165</v>
       </c>
-      <c r="Z2" s="5">
+      <c r="AA2" s="5">
         <v>12129151158</v>
       </c>
-      <c r="AA2" s="5">
+      <c r="AB2" s="5">
         <v>79232794237</v>
       </c>
-      <c r="AB2" t="s">
-        <v>148</v>
-      </c>
-      <c r="AC2" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="AD2" t="s">
-        <v>159</v>
-      </c>
-      <c r="AE2" s="2" t="s">
+      <c r="AC2" t="s">
+        <v>147</v>
+      </c>
+      <c r="AD2" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>158</v>
+      </c>
+      <c r="AF2" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="AF2" s="2" t="s">
+      <c r="AG2" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="AG2" s="5">
+      <c r="AH2" s="5">
         <v>1915</v>
       </c>
-      <c r="AH2" s="5">
+      <c r="AI2" s="5">
         <v>707553</v>
       </c>
-      <c r="AI2" s="5">
+      <c r="AJ2" s="5">
         <v>23163683192</v>
       </c>
-      <c r="AJ2" s="5">
+      <c r="AK2" s="5">
         <v>79966151614</v>
       </c>
-      <c r="AK2" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="AL2" s="5" t="s">
+      <c r="AL2" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="AM2" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="AM2" s="2">
-        <v>3</v>
-      </c>
       <c r="AN2" s="2">
-        <v>55</v>
+        <v>4</v>
       </c>
       <c r="AO2" s="2">
+        <v>101</v>
+      </c>
+      <c r="AP2" s="2">
         <v>8</v>
       </c>
-      <c r="AP2" s="2">
+      <c r="AQ2" s="2">
         <v>2</v>
       </c>
-      <c r="AQ2" s="9">
-        <v>70</v>
-      </c>
-      <c r="AR2" s="2" t="s">
+      <c r="AR2" s="7">
+        <v>70</v>
+      </c>
+      <c r="AS2" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="AS2" s="2" t="s">
-        <v>69</v>
-      </c>
       <c r="AT2" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="AU2" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="AU2" s="2" t="s">
+      <c r="AV2" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="AV2" s="2" t="s">
-        <v>74</v>
-      </c>
       <c r="AW2" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="AX2" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="AX2" s="9">
+      <c r="AY2" s="7">
         <v>3397819</v>
       </c>
-      <c r="AY2" s="2">
-        <v>74</v>
-      </c>
-      <c r="AZ2" s="2">
-        <v>1978</v>
-      </c>
-      <c r="BA2" s="2">
+      <c r="AZ2" s="10">
+        <v>96</v>
+      </c>
+      <c r="BA2" s="13" t="s">
+        <v>195</v>
+      </c>
+      <c r="BB2" s="11">
         <v>12</v>
       </c>
-      <c r="BB2" s="2">
+      <c r="BC2" s="2">
         <v>4</v>
       </c>
-      <c r="BC2" s="2" t="s">
-        <v>69</v>
-      </c>
       <c r="BD2" s="2" t="s">
         <v>69</v>
       </c>
       <c r="BE2" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="BF2" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="BF2" s="2" t="s">
+      <c r="BG2" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="BG2" s="2" t="s">
+      <c r="BH2" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="BH2" s="2">
+      <c r="BI2" s="2">
         <v>23</v>
       </c>
-      <c r="BI2" s="9" t="s">
+      <c r="BJ2" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="BJ2" s="2">
+      <c r="BK2" s="2">
         <v>3.46</v>
       </c>
-      <c r="BK2" s="2" t="s">
+      <c r="BL2" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="BL2" s="2" t="s">
-        <v>69</v>
-      </c>
       <c r="BM2" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="BN2" s="2" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="3" spans="1:65" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:66">
       <c r="A3" s="2" t="s">
         <v>74</v>
       </c>
@@ -1487,7 +1607,7 @@
         <v>35000</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>69</v>
@@ -1514,7 +1634,7 @@
         <v>45</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="P3" s="2">
         <v>1903</v>
@@ -1522,39 +1642,39 @@
       <c r="Q3" s="2">
         <v>580301</v>
       </c>
-      <c r="R3" s="7">
+      <c r="R3" s="5">
         <v>71653031154</v>
       </c>
-      <c r="S3" s="7">
+      <c r="S3" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="T3" s="5">
         <v>79807206751</v>
       </c>
-      <c r="T3" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="U3" s="9" t="s">
+      <c r="U3" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="V3" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="V3" s="2" t="s">
-        <v>161</v>
-      </c>
       <c r="W3" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="X3" s="5">
+        <v>160</v>
+      </c>
+      <c r="X3" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="Y3" s="5">
         <v>1920</v>
       </c>
-      <c r="Y3" s="4">
+      <c r="Z3" s="4">
         <v>632800</v>
       </c>
-      <c r="Z3" s="4">
+      <c r="AA3" s="4">
         <v>70838605618</v>
       </c>
-      <c r="AA3" s="4">
+      <c r="AB3" s="4">
         <v>79466194497</v>
       </c>
-      <c r="AB3" s="2" t="s">
-        <v>74</v>
-      </c>
       <c r="AC3" s="2" t="s">
         <v>74</v>
       </c>
@@ -1567,7 +1687,7 @@
       <c r="AF3" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="AG3" s="5" t="s">
+      <c r="AG3" s="2" t="s">
         <v>74</v>
       </c>
       <c r="AH3" s="5" t="s">
@@ -1579,100 +1699,103 @@
       <c r="AJ3" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="AK3" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="AL3" s="5" t="s">
+      <c r="AK3" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="AL3" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="AM3" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="AM3" s="2">
+      <c r="AN3" s="2">
         <v>5</v>
       </c>
-      <c r="AN3" s="2">
+      <c r="AO3" s="2">
         <v>102</v>
-      </c>
-      <c r="AO3" s="2">
-        <v>3</v>
       </c>
       <c r="AP3" s="2">
         <v>3</v>
       </c>
-      <c r="AQ3" s="9">
+      <c r="AQ3" s="2">
+        <v>3</v>
+      </c>
+      <c r="AR3" s="7">
         <v>80</v>
       </c>
-      <c r="AR3" s="2" t="s">
+      <c r="AS3" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="AS3" t="s">
-        <v>69</v>
-      </c>
-      <c r="AT3" s="2" t="s">
+      <c r="AT3" t="s">
+        <v>69</v>
+      </c>
+      <c r="AU3" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="AU3" s="2" t="s">
+      <c r="AV3" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="AV3" s="2" t="s">
-        <v>74</v>
-      </c>
       <c r="AW3" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="AX3" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="AX3" s="9">
+      <c r="AY3" s="7">
         <v>4246742</v>
       </c>
-      <c r="AY3" s="2">
+      <c r="AZ3" s="10">
         <v>27</v>
       </c>
-      <c r="AZ3" s="2">
-        <v>1982</v>
-      </c>
-      <c r="BA3" s="2">
+      <c r="BA3" s="13" t="s">
+        <v>185</v>
+      </c>
+      <c r="BB3" s="11">
         <v>9</v>
       </c>
-      <c r="BB3" s="2">
+      <c r="BC3" s="2">
         <v>5</v>
       </c>
-      <c r="BC3" s="2" t="s">
-        <v>69</v>
-      </c>
       <c r="BD3" s="2" t="s">
         <v>69</v>
       </c>
       <c r="BE3" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="BF3" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="BF3" s="2" t="s">
+      <c r="BG3" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="BG3" s="2" t="s">
+      <c r="BH3" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="BH3" s="2">
+      <c r="BI3" s="2">
         <v>13</v>
       </c>
-      <c r="BI3" s="9" t="s">
+      <c r="BJ3" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="BJ3" s="2">
+      <c r="BK3" s="2">
         <v>2.82</v>
       </c>
-      <c r="BK3" s="2" t="s">
+      <c r="BL3" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="BL3" s="2" t="s">
-        <v>69</v>
-      </c>
       <c r="BM3" s="2" t="s">
         <v>69</v>
       </c>
+      <c r="BN3" s="2" t="s">
+        <v>69</v>
+      </c>
     </row>
-    <row r="4" spans="1:65" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:66">
       <c r="A4" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C4" s="2">
         <v>56000</v>
@@ -1684,7 +1807,7 @@
         <v>56000</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>70</v>
@@ -1711,7 +1834,7 @@
         <v>30</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="P4" s="2">
         <v>1907</v>
@@ -1719,157 +1842,160 @@
       <c r="Q4" s="2">
         <v>570691</v>
       </c>
-      <c r="R4" s="7">
+      <c r="R4" s="5">
         <v>33266613098</v>
       </c>
-      <c r="S4" s="7">
+      <c r="S4" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="T4" s="5">
         <v>79236003943</v>
       </c>
-      <c r="T4" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="U4" s="9" t="s">
+      <c r="U4" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="V4" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="V4" s="2" t="s">
-        <v>162</v>
-      </c>
       <c r="W4" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="X4" s="4">
+        <v>161</v>
+      </c>
+      <c r="X4" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="Y4" s="4">
         <v>1904</v>
       </c>
-      <c r="Y4" s="11">
+      <c r="Z4" s="8">
         <v>746789</v>
       </c>
-      <c r="Z4" s="5">
+      <c r="AA4" s="5">
         <v>15603313658</v>
       </c>
-      <c r="AA4" s="5">
+      <c r="AB4" s="5">
         <v>79685258072</v>
       </c>
-      <c r="AB4" t="s">
-        <v>149</v>
-      </c>
-      <c r="AC4" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="AD4" t="s">
-        <v>155</v>
-      </c>
-      <c r="AE4" s="2" t="s">
+      <c r="AC4" t="s">
+        <v>148</v>
+      </c>
+      <c r="AD4" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="AE4" t="s">
+        <v>154</v>
+      </c>
+      <c r="AF4" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="AF4" s="2" t="s">
+      <c r="AG4" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="AG4" s="4">
+      <c r="AH4" s="4">
         <v>1913</v>
       </c>
-      <c r="AH4" s="5">
+      <c r="AI4" s="5">
         <v>350147</v>
       </c>
-      <c r="AI4" s="5">
+      <c r="AJ4" s="5">
         <v>41814943016</v>
       </c>
-      <c r="AJ4" s="5">
+      <c r="AK4" s="5">
         <v>79466353077</v>
       </c>
-      <c r="AK4" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="AL4" s="5" t="s">
+      <c r="AL4" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="AM4" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="AM4" s="2">
+      <c r="AN4" s="2">
         <v>2</v>
       </c>
-      <c r="AN4" s="2">
+      <c r="AO4" s="2">
         <v>31</v>
       </c>
-      <c r="AO4" s="2">
+      <c r="AP4" s="2">
         <v>7</v>
       </c>
-      <c r="AP4" s="2">
+      <c r="AQ4" s="2">
         <v>4</v>
       </c>
-      <c r="AQ4" s="9">
+      <c r="AR4" s="7">
         <v>100</v>
       </c>
-      <c r="AR4" s="2" t="s">
+      <c r="AS4" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="AS4" s="2" t="s">
-        <v>69</v>
-      </c>
       <c r="AT4" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="AU4" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="AU4" s="2" t="s">
+      <c r="AV4" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="AV4" s="2" t="s">
-        <v>74</v>
-      </c>
       <c r="AW4" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="AX4" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="AX4" s="9">
+      <c r="AY4" s="7">
         <v>4909056</v>
       </c>
-      <c r="AY4" s="2">
+      <c r="AZ4" s="10">
         <v>12</v>
       </c>
-      <c r="AZ4" s="2">
-        <v>2012</v>
-      </c>
-      <c r="BA4" s="2">
+      <c r="BA4" s="13" t="s">
+        <v>186</v>
+      </c>
+      <c r="BB4" s="11">
         <v>9</v>
       </c>
-      <c r="BB4" s="2">
+      <c r="BC4" s="2">
         <v>4</v>
       </c>
-      <c r="BC4" s="2" t="s">
-        <v>69</v>
-      </c>
       <c r="BD4" s="2" t="s">
         <v>69</v>
       </c>
       <c r="BE4" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="BF4" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="BF4" s="2" t="s">
+      <c r="BG4" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="BG4" s="2" t="s">
+      <c r="BH4" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="BH4" s="2">
+      <c r="BI4" s="2">
         <v>4</v>
       </c>
-      <c r="BI4" s="9" t="s">
+      <c r="BJ4" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="BJ4" s="2">
+      <c r="BK4" s="2">
         <v>5.03</v>
       </c>
-      <c r="BK4" s="2" t="s">
+      <c r="BL4" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="BL4" s="2" t="s">
-        <v>69</v>
-      </c>
       <c r="BM4" s="2" t="s">
         <v>69</v>
       </c>
+      <c r="BN4" s="2" t="s">
+        <v>69</v>
+      </c>
     </row>
-    <row r="5" spans="1:65" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:66">
       <c r="A5" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C5" s="2">
         <v>23000</v>
@@ -1881,7 +2007,7 @@
         <v>28000</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>69</v>
@@ -1908,7 +2034,7 @@
         <v>60</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="P5" s="2">
         <v>1911</v>
@@ -1916,152 +2042,155 @@
       <c r="Q5" s="2">
         <v>170595</v>
       </c>
-      <c r="R5" s="7">
+      <c r="R5" s="5">
         <v>68261558356</v>
       </c>
-      <c r="S5" s="7">
+      <c r="S5" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="T5" s="5">
         <v>79641863919</v>
       </c>
-      <c r="T5" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="U5" s="9" t="s">
+      <c r="U5" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="V5" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="V5" s="2" t="s">
-        <v>162</v>
-      </c>
       <c r="W5" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="X5" s="4">
+        <v>161</v>
+      </c>
+      <c r="X5" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="Y5" s="4">
         <v>1904</v>
       </c>
-      <c r="Y5" s="11">
+      <c r="Z5" s="8">
         <v>746789</v>
       </c>
-      <c r="Z5" s="5">
+      <c r="AA5" s="5">
         <v>15603313658</v>
       </c>
-      <c r="AA5" s="5">
+      <c r="AB5" s="5">
         <v>79685258072</v>
       </c>
-      <c r="AB5" t="s">
-        <v>150</v>
-      </c>
-      <c r="AC5" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="AD5" t="s">
-        <v>156</v>
-      </c>
-      <c r="AE5" s="2" t="s">
+      <c r="AC5" t="s">
+        <v>149</v>
+      </c>
+      <c r="AD5" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="AE5" t="s">
+        <v>155</v>
+      </c>
+      <c r="AF5" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="AF5" s="2" t="s">
+      <c r="AG5" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="AG5" s="4">
+      <c r="AH5" s="4">
         <v>1912</v>
       </c>
-      <c r="AH5" s="5">
+      <c r="AI5" s="5">
         <v>708165</v>
       </c>
-      <c r="AI5" s="5">
+      <c r="AJ5" s="5">
         <v>36125690516</v>
       </c>
-      <c r="AJ5" s="5">
+      <c r="AK5" s="5">
         <v>79473995064</v>
       </c>
-      <c r="AK5" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="AL5" s="5" t="s">
+      <c r="AL5" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="AM5" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="AM5" s="2">
+      <c r="AN5" s="2">
         <v>1</v>
       </c>
-      <c r="AN5" s="2">
+      <c r="AO5" s="2">
         <v>14</v>
       </c>
-      <c r="AO5" s="2">
+      <c r="AP5" s="2">
         <v>4</v>
       </c>
-      <c r="AP5" s="13">
+      <c r="AQ5" s="2">
         <v>2</v>
       </c>
-      <c r="AQ5" s="9">
+      <c r="AR5" s="7">
         <v>65</v>
       </c>
-      <c r="AR5" s="2" t="s">
+      <c r="AS5" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="AS5" s="2" t="s">
-        <v>70</v>
-      </c>
       <c r="AT5" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="AU5" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="AU5" s="2" t="s">
+      <c r="AV5" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="AV5" s="2">
+      <c r="AW5" s="2">
         <v>56126.8</v>
       </c>
-      <c r="AW5" s="2" t="s">
+      <c r="AX5" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="AX5" s="9">
+      <c r="AY5" s="7">
         <v>3827260</v>
       </c>
-      <c r="AY5" s="2">
+      <c r="AZ5" s="10">
         <v>23</v>
       </c>
-      <c r="AZ5" s="2">
-        <v>1964</v>
-      </c>
-      <c r="BA5" s="2">
+      <c r="BA5" s="13" t="s">
+        <v>187</v>
+      </c>
+      <c r="BB5" s="11">
         <v>5</v>
       </c>
-      <c r="BB5" s="2">
+      <c r="BC5" s="2">
         <v>3</v>
       </c>
-      <c r="BC5" s="2" t="s">
-        <v>70</v>
-      </c>
       <c r="BD5" s="2" t="s">
         <v>70</v>
       </c>
       <c r="BE5" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="BF5" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="BF5" s="2" t="s">
+      <c r="BG5" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="BG5" s="2" t="s">
+      <c r="BH5" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="BH5" s="13">
+      <c r="BI5" s="2">
         <v>20</v>
       </c>
-      <c r="BI5" s="9" t="s">
+      <c r="BJ5" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="BJ5" s="2">
+      <c r="BK5" s="2">
         <v>3.84</v>
       </c>
-      <c r="BK5" s="2" t="s">
+      <c r="BL5" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="BL5" s="2" t="s">
-        <v>70</v>
-      </c>
       <c r="BM5" s="2" t="s">
         <v>70</v>
       </c>
+      <c r="BN5" s="2" t="s">
+        <v>70</v>
+      </c>
     </row>
-    <row r="6" spans="1:65" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:66">
       <c r="A6" s="2" t="s">
         <v>74</v>
       </c>
@@ -2078,7 +2207,7 @@
         <v>25000</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>69</v>
@@ -2105,7 +2234,7 @@
         <v>40</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="P6" s="2">
         <v>1915</v>
@@ -2113,39 +2242,39 @@
       <c r="Q6" s="2">
         <v>935593</v>
       </c>
-      <c r="R6" s="7">
+      <c r="R6" s="5">
         <v>59406567729</v>
       </c>
-      <c r="S6" s="7">
+      <c r="S6" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="T6" s="5">
         <v>79809334527</v>
       </c>
-      <c r="T6" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="U6" s="9" t="s">
+      <c r="U6" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="V6" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="V6" s="2" t="s">
-        <v>161</v>
-      </c>
       <c r="W6" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="X6" s="5">
+        <v>160</v>
+      </c>
+      <c r="X6" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="Y6" s="5">
         <v>1920</v>
       </c>
-      <c r="Y6" s="4">
+      <c r="Z6" s="4">
         <v>632800</v>
       </c>
-      <c r="Z6" s="5">
+      <c r="AA6" s="5">
         <v>22868427778</v>
       </c>
-      <c r="AA6" s="5">
+      <c r="AB6" s="5">
         <v>79665769974</v>
       </c>
-      <c r="AB6" s="2" t="s">
-        <v>74</v>
-      </c>
       <c r="AC6" s="2" t="s">
         <v>74</v>
       </c>
@@ -2158,10 +2287,10 @@
       <c r="AF6" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="AG6" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="AH6" s="5" t="s">
+      <c r="AG6" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="AH6" s="4" t="s">
         <v>74</v>
       </c>
       <c r="AI6" s="5" t="s">
@@ -2170,95 +2299,98 @@
       <c r="AJ6" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="AK6" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="AL6" s="5" t="s">
+      <c r="AK6" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="AL6" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="AM6" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="AM6" s="2">
+      <c r="AN6" s="2">
         <v>2</v>
       </c>
-      <c r="AN6" s="2">
+      <c r="AO6" s="2">
         <v>24</v>
-      </c>
-      <c r="AO6" s="2">
-        <v>2</v>
       </c>
       <c r="AP6" s="2">
         <v>2</v>
       </c>
-      <c r="AQ6" s="9">
+      <c r="AQ6" s="2">
+        <v>2</v>
+      </c>
+      <c r="AR6" s="7">
         <v>47</v>
       </c>
-      <c r="AR6" s="2" t="s">
+      <c r="AS6" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="AS6" s="2" t="s">
-        <v>70</v>
-      </c>
       <c r="AT6" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="AU6" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="AU6" s="2" t="s">
+      <c r="AV6" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="AV6" s="2">
+      <c r="AW6" s="2">
         <v>0</v>
       </c>
-      <c r="AW6" s="2" t="s">
+      <c r="AX6" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="AX6" s="9">
+      <c r="AY6" s="7">
         <v>2555172</v>
       </c>
-      <c r="AY6" s="2" t="s">
+      <c r="AZ6" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="AZ6" s="2">
-        <v>1959</v>
-      </c>
-      <c r="BA6" s="2">
+      <c r="BA6" s="13" t="s">
+        <v>188</v>
+      </c>
+      <c r="BB6" s="11">
         <v>5</v>
       </c>
-      <c r="BB6" s="2">
+      <c r="BC6" s="2">
         <v>4</v>
       </c>
-      <c r="BC6" s="2" t="s">
-        <v>70</v>
-      </c>
       <c r="BD6" s="2" t="s">
         <v>70</v>
       </c>
       <c r="BE6" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="BF6" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="BF6" s="2" t="s">
+      <c r="BG6" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="BG6" s="2" t="s">
+      <c r="BH6" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="BH6" s="2">
+      <c r="BI6" s="2">
         <v>24</v>
       </c>
-      <c r="BI6" s="9" t="s">
+      <c r="BJ6" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="BJ6" s="2">
+      <c r="BK6" s="2">
         <v>4.13</v>
       </c>
-      <c r="BK6" s="2" t="s">
+      <c r="BL6" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="BL6" s="2" t="s">
-        <v>69</v>
-      </c>
       <c r="BM6" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="BN6" s="2" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="7" spans="1:65" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:66">
       <c r="A7" s="2" t="s">
         <v>74</v>
       </c>
@@ -2275,7 +2407,7 @@
         <v>31000</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>69</v>
@@ -2302,7 +2434,7 @@
         <v>40</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="P7" s="2">
         <v>1914</v>
@@ -2310,39 +2442,39 @@
       <c r="Q7" s="2">
         <v>315512</v>
       </c>
-      <c r="R7" s="7">
+      <c r="R7" s="5">
         <v>87745672288</v>
       </c>
-      <c r="S7" s="7">
+      <c r="S7" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="T7" s="5">
         <v>79463637760</v>
       </c>
-      <c r="T7" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="U7" s="9" t="s">
+      <c r="U7" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="V7" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="V7" s="2" t="s">
+      <c r="W7" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="X7" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="W7" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="X7" s="4">
+      <c r="Y7" s="4">
         <v>1916</v>
       </c>
-      <c r="Y7" s="11">
+      <c r="Z7" s="8">
         <v>705814</v>
       </c>
-      <c r="Z7" s="5">
+      <c r="AA7" s="5">
         <v>19353775566</v>
       </c>
-      <c r="AA7" s="5">
+      <c r="AB7" s="5">
         <v>79145411713</v>
       </c>
-      <c r="AB7" s="2" t="s">
-        <v>74</v>
-      </c>
       <c r="AC7" s="2" t="s">
         <v>74</v>
       </c>
@@ -2355,10 +2487,10 @@
       <c r="AF7" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="AG7" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="AH7" s="5" t="s">
+      <c r="AG7" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="AH7" s="4" t="s">
         <v>74</v>
       </c>
       <c r="AI7" s="5" t="s">
@@ -2367,95 +2499,98 @@
       <c r="AJ7" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="AK7" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="AL7" s="5" t="s">
+      <c r="AK7" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="AL7" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="AM7" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="AM7" s="2">
+      <c r="AN7" s="2">
         <v>4</v>
       </c>
-      <c r="AN7" s="2">
+      <c r="AO7" s="2">
         <v>130</v>
       </c>
-      <c r="AO7" s="2">
+      <c r="AP7" s="2">
         <v>6</v>
       </c>
-      <c r="AP7" s="2">
+      <c r="AQ7" s="2">
         <v>3</v>
       </c>
-      <c r="AQ7" s="9">
+      <c r="AR7" s="7">
         <v>65</v>
       </c>
-      <c r="AR7" s="2" t="s">
+      <c r="AS7" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="AS7" s="2" t="s">
-        <v>70</v>
-      </c>
       <c r="AT7" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="AU7" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="AU7" s="2" t="s">
+      <c r="AV7" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="AV7" s="2" t="s">
-        <v>74</v>
-      </c>
       <c r="AW7" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="AX7" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="AX7" s="9">
+      <c r="AY7" s="7">
         <v>4454951</v>
       </c>
-      <c r="AY7" s="2">
+      <c r="AZ7" s="10">
         <v>18</v>
       </c>
-      <c r="AZ7" s="2">
-        <v>1981</v>
-      </c>
-      <c r="BA7" s="2">
+      <c r="BA7" s="13" t="s">
+        <v>189</v>
+      </c>
+      <c r="BB7" s="11">
         <v>9</v>
       </c>
-      <c r="BB7" s="2">
+      <c r="BC7" s="2">
         <v>4</v>
       </c>
-      <c r="BC7" s="2" t="s">
-        <v>69</v>
-      </c>
       <c r="BD7" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="BE7" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="BF7" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="BF7" s="2" t="s">
+      <c r="BG7" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="BG7" s="2" t="s">
+      <c r="BH7" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="BH7" s="2">
+      <c r="BI7" s="2">
         <v>15</v>
       </c>
-      <c r="BI7" s="3" t="s">
+      <c r="BJ7" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="BJ7" s="2">
+      <c r="BK7" s="2">
         <v>5.01</v>
       </c>
-      <c r="BK7" s="2" t="s">
+      <c r="BL7" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="BL7" s="2" t="s">
-        <v>70</v>
-      </c>
       <c r="BM7" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="BN7" s="2" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="8" spans="1:65" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:66">
       <c r="A8" s="2" t="s">
         <v>74</v>
       </c>
@@ -2472,7 +2607,7 @@
         <v>24000</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>70</v>
@@ -2499,7 +2634,7 @@
         <v>45</v>
       </c>
       <c r="O8" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="P8" s="2">
         <v>1911</v>
@@ -2507,39 +2642,39 @@
       <c r="Q8" s="2">
         <v>177558</v>
       </c>
-      <c r="R8" s="7">
+      <c r="R8" s="5">
         <v>67504839581</v>
       </c>
-      <c r="S8" s="7">
+      <c r="S8" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="T8" s="5">
         <v>79874043664</v>
       </c>
-      <c r="T8" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="U8" s="9" t="s">
+      <c r="U8" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="V8" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="V8" s="2" t="s">
-        <v>160</v>
-      </c>
       <c r="W8" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="X8" s="5">
+        <v>159</v>
+      </c>
+      <c r="X8" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="Y8" s="5">
         <v>1925</v>
       </c>
-      <c r="Y8" s="4">
+      <c r="Z8" s="4">
         <v>570165</v>
       </c>
-      <c r="Z8" s="5">
+      <c r="AA8" s="5">
         <v>12129151158</v>
       </c>
-      <c r="AA8" s="5">
+      <c r="AB8" s="5">
         <v>79232794237</v>
       </c>
-      <c r="AB8" s="2" t="s">
-        <v>74</v>
-      </c>
       <c r="AC8" s="2" t="s">
         <v>74</v>
       </c>
@@ -2547,15 +2682,15 @@
         <v>74</v>
       </c>
       <c r="AE8" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="AF8" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="AF8" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="AG8" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="AH8" s="5" t="s">
+      <c r="AG8" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="AH8" s="4" t="s">
         <v>74</v>
       </c>
       <c r="AI8" s="5" t="s">
@@ -2564,100 +2699,103 @@
       <c r="AJ8" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="AK8" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="AL8" s="5" t="s">
+      <c r="AK8" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="AL8" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="AM8" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="AM8" s="2">
+      <c r="AN8" s="2">
         <v>3</v>
       </c>
-      <c r="AN8" s="2">
+      <c r="AO8" s="2">
         <v>81</v>
       </c>
-      <c r="AO8" s="2">
+      <c r="AP8" s="2">
         <v>3</v>
       </c>
-      <c r="AP8" s="2">
+      <c r="AQ8" s="2">
         <v>2</v>
       </c>
-      <c r="AQ8" s="2">
+      <c r="AR8" s="2">
         <v>60</v>
       </c>
-      <c r="AR8" s="2" t="s">
+      <c r="AS8" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="AS8" s="2" t="s">
-        <v>70</v>
-      </c>
       <c r="AT8" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="AU8" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="AU8" s="2" t="s">
+      <c r="AV8" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="AV8" s="2">
+      <c r="AW8" s="2">
         <v>0</v>
       </c>
-      <c r="AW8" s="2" t="s">
+      <c r="AX8" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="AX8" s="9">
+      <c r="AY8" s="7">
         <v>3036872</v>
       </c>
-      <c r="AY8" s="2">
+      <c r="AZ8" s="10">
         <v>39</v>
       </c>
-      <c r="AZ8" s="2">
-        <v>1967</v>
-      </c>
-      <c r="BA8" s="2">
+      <c r="BA8" s="13" t="s">
+        <v>190</v>
+      </c>
+      <c r="BB8" s="11">
         <v>5</v>
       </c>
-      <c r="BB8" s="2">
+      <c r="BC8" s="2">
         <v>4</v>
       </c>
-      <c r="BC8" s="2" t="s">
-        <v>70</v>
-      </c>
       <c r="BD8" s="2" t="s">
         <v>70</v>
       </c>
       <c r="BE8" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="BF8" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="BF8" s="2" t="s">
+      <c r="BG8" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="BG8" s="2" t="s">
+      <c r="BH8" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="BH8" s="2">
+      <c r="BI8" s="2">
         <v>37</v>
       </c>
-      <c r="BI8" s="9" t="s">
+      <c r="BJ8" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="BJ8" s="8">
+      <c r="BK8" s="6">
         <v>2.56</v>
       </c>
-      <c r="BK8" s="2" t="s">
+      <c r="BL8" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="BL8" s="2" t="s">
-        <v>70</v>
-      </c>
       <c r="BM8" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="BN8" s="2" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="9" spans="1:65" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:66" ht="17.100000000000001" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C9" s="2">
         <v>43000</v>
@@ -2669,7 +2807,7 @@
         <v>45000</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>70</v>
@@ -2696,7 +2834,7 @@
         <v>30</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P9" s="2">
         <v>1915</v>
@@ -2704,157 +2842,160 @@
       <c r="Q9" s="2">
         <v>991173</v>
       </c>
-      <c r="R9" s="6">
+      <c r="R9" s="4">
         <v>35642877954</v>
       </c>
-      <c r="S9" s="7">
+      <c r="S9" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="T9" s="5">
         <v>79602775769</v>
       </c>
-      <c r="T9" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="U9" s="9" t="s">
+      <c r="U9" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="V9" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="V9" s="2" t="s">
+      <c r="W9" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="X9" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="W9" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="X9" s="4">
+      <c r="Y9" s="4">
         <v>1916</v>
       </c>
-      <c r="Y9" s="11">
+      <c r="Z9" s="8">
         <v>705814</v>
       </c>
-      <c r="Z9" s="5">
+      <c r="AA9" s="5">
         <v>19353775566</v>
       </c>
-      <c r="AA9" s="5">
+      <c r="AB9" s="5">
         <v>79145411713</v>
       </c>
-      <c r="AB9" s="2" t="s">
-        <v>151</v>
-      </c>
       <c r="AC9" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="AD9" t="s">
-        <v>157</v>
-      </c>
-      <c r="AE9" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="AD9" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="AE9" t="s">
+        <v>156</v>
+      </c>
+      <c r="AF9" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="AF9" s="2" t="s">
+      <c r="AG9" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="AG9" s="4">
+      <c r="AH9" s="4">
         <v>1915</v>
       </c>
-      <c r="AH9" s="5">
+      <c r="AI9" s="5">
         <v>476677</v>
       </c>
-      <c r="AI9" s="5">
+      <c r="AJ9" s="5">
         <v>33844350786</v>
       </c>
-      <c r="AJ9" s="12">
+      <c r="AK9" s="9">
         <v>79348959710</v>
       </c>
-      <c r="AK9" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="AL9" s="5" t="s">
+      <c r="AL9" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="AM9" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="AM9" s="2">
+      <c r="AN9" s="2">
         <v>1</v>
       </c>
-      <c r="AN9" s="2">
+      <c r="AO9" s="2">
         <v>24</v>
-      </c>
-      <c r="AO9" s="2">
-        <v>4</v>
       </c>
       <c r="AP9" s="2">
         <v>4</v>
       </c>
-      <c r="AQ9" s="9">
+      <c r="AQ9" s="2">
+        <v>4</v>
+      </c>
+      <c r="AR9" s="7">
         <v>94</v>
       </c>
-      <c r="AR9" s="2" t="s">
+      <c r="AS9" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="AS9" s="2" t="s">
-        <v>69</v>
-      </c>
       <c r="AT9" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="AU9" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="AU9" s="2" t="s">
+      <c r="AV9" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="AV9" s="2" t="s">
-        <v>74</v>
-      </c>
       <c r="AW9" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="AX9" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="AX9" s="9">
+      <c r="AY9" s="7">
         <v>4090021</v>
       </c>
-      <c r="AY9" s="2">
+      <c r="AZ9" s="10">
         <v>19</v>
       </c>
-      <c r="AZ9" s="2">
-        <v>2015</v>
-      </c>
-      <c r="BA9" s="2">
+      <c r="BA9" s="13" t="s">
+        <v>191</v>
+      </c>
+      <c r="BB9" s="11">
         <v>5</v>
       </c>
-      <c r="BB9" s="2">
+      <c r="BC9" s="2">
         <v>7</v>
       </c>
-      <c r="BC9" s="2" t="s">
-        <v>70</v>
-      </c>
       <c r="BD9" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="BE9" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="BF9" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="BF9" s="2" t="s">
+      <c r="BG9" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="BG9" s="2" t="s">
+      <c r="BH9" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="BH9" s="2">
+      <c r="BI9" s="2">
         <v>12</v>
       </c>
-      <c r="BI9" s="9" t="s">
+      <c r="BJ9" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="BJ9" s="2">
+      <c r="BK9" s="2">
         <v>2.82</v>
       </c>
-      <c r="BK9" s="2" t="s">
+      <c r="BL9" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="BL9" s="2" t="s">
-        <v>70</v>
-      </c>
       <c r="BM9" s="2" t="s">
         <v>70</v>
       </c>
+      <c r="BN9" s="2" t="s">
+        <v>70</v>
+      </c>
     </row>
-    <row r="10" spans="1:65" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:66">
       <c r="A10" s="2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C10" s="2">
         <v>21500</v>
@@ -2866,7 +3007,7 @@
         <v>23000</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>69</v>
@@ -2893,7 +3034,7 @@
         <v>45</v>
       </c>
       <c r="O10" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="P10" s="2">
         <v>1915</v>
@@ -2901,152 +3042,155 @@
       <c r="Q10" s="2">
         <v>230801</v>
       </c>
-      <c r="R10" s="7">
+      <c r="R10" s="5">
         <v>18205896570</v>
       </c>
-      <c r="S10" s="7">
+      <c r="S10" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="T10" s="5">
         <v>79874291979</v>
       </c>
-      <c r="T10" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="U10" s="9" t="s">
+      <c r="U10" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="V10" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="V10" s="2" t="s">
-        <v>162</v>
-      </c>
       <c r="W10" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="X10" s="4">
+        <v>161</v>
+      </c>
+      <c r="X10" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="Y10" s="4">
         <v>1904</v>
       </c>
-      <c r="Y10" s="11">
+      <c r="Z10" s="8">
         <v>746789</v>
       </c>
-      <c r="Z10" s="5">
+      <c r="AA10" s="5">
         <v>15603313658</v>
       </c>
-      <c r="AA10" s="5">
+      <c r="AB10" s="5">
         <v>79685258072</v>
       </c>
-      <c r="AB10" t="s">
+      <c r="AC10" t="s">
+        <v>151</v>
+      </c>
+      <c r="AD10" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="AC10" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="AD10" t="s">
-        <v>158</v>
-      </c>
-      <c r="AE10" s="2" t="s">
+      <c r="AE10" t="s">
+        <v>157</v>
+      </c>
+      <c r="AF10" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="AF10" s="2" t="s">
+      <c r="AG10" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="AG10" s="10">
+      <c r="AH10" s="4">
         <v>1903</v>
       </c>
-      <c r="AH10" s="5">
+      <c r="AI10" s="5">
         <v>663847</v>
       </c>
-      <c r="AI10" s="5">
+      <c r="AJ10" s="5">
         <v>98342318654</v>
       </c>
-      <c r="AJ10" s="5">
+      <c r="AK10" s="5">
         <v>79609569765</v>
       </c>
-      <c r="AK10" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="AL10" s="4" t="s">
+      <c r="AL10" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="AM10" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="AM10" s="2">
+      <c r="AN10" s="2">
         <v>2</v>
       </c>
-      <c r="AN10" s="2">
+      <c r="AO10" s="2">
         <v>38</v>
       </c>
-      <c r="AO10" s="2">
+      <c r="AP10" s="2">
         <v>5</v>
       </c>
-      <c r="AP10" s="2">
+      <c r="AQ10" s="2">
         <v>2</v>
       </c>
-      <c r="AQ10" s="9">
+      <c r="AR10" s="7">
         <v>71</v>
       </c>
-      <c r="AR10" s="2" t="s">
+      <c r="AS10" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="AS10" s="2" t="s">
-        <v>69</v>
-      </c>
       <c r="AT10" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="AU10" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="AU10" s="2" t="s">
+      <c r="AV10" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="AV10" s="2">
+      <c r="AW10" s="2">
         <v>34690.370000000003</v>
       </c>
-      <c r="AW10" s="2" t="s">
+      <c r="AX10" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="AX10" s="9">
+      <c r="AY10" s="7">
         <v>3944155</v>
       </c>
-      <c r="AY10" s="2">
+      <c r="AZ10" s="10">
         <v>24</v>
       </c>
-      <c r="AZ10" s="2">
-        <v>1970</v>
-      </c>
-      <c r="BA10" s="2">
+      <c r="BA10" s="13" t="s">
+        <v>192</v>
+      </c>
+      <c r="BB10" s="11">
         <v>5</v>
       </c>
-      <c r="BB10" s="2">
+      <c r="BC10" s="2">
         <v>4</v>
       </c>
-      <c r="BC10" s="2" t="s">
-        <v>70</v>
-      </c>
       <c r="BD10" s="2" t="s">
         <v>70</v>
       </c>
       <c r="BE10" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="BF10" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="BF10" s="2" t="s">
+      <c r="BG10" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="BG10" s="2" t="s">
+      <c r="BH10" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="BH10" s="2">
+      <c r="BI10" s="2">
         <v>43</v>
       </c>
-      <c r="BI10" s="9" t="s">
+      <c r="BJ10" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="BJ10" s="2">
+      <c r="BK10" s="2">
         <v>0.84</v>
       </c>
-      <c r="BK10" s="2" t="s">
+      <c r="BL10" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="BL10" s="2" t="s">
-        <v>69</v>
-      </c>
       <c r="BM10" s="2" t="s">
         <v>69</v>
       </c>
+      <c r="BN10" s="2" t="s">
+        <v>69</v>
+      </c>
     </row>
-    <row r="11" spans="1:65" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:66">
       <c r="A11" s="2" t="s">
         <v>74</v>
       </c>
@@ -3063,7 +3207,7 @@
         <v>38000</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>69</v>
@@ -3090,7 +3234,7 @@
         <v>60</v>
       </c>
       <c r="O11" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="P11" s="2">
         <v>1911</v>
@@ -3098,39 +3242,39 @@
       <c r="Q11" s="2">
         <v>629151</v>
       </c>
-      <c r="R11" s="7">
+      <c r="R11" s="5">
         <v>34928998673</v>
       </c>
-      <c r="S11" s="6">
+      <c r="S11" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="T11" s="4">
         <v>79409766923</v>
       </c>
-      <c r="T11" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="U11" s="9" t="s">
+      <c r="U11" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="V11" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="V11" s="2" t="s">
-        <v>161</v>
-      </c>
       <c r="W11" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="X11" s="5">
+        <v>160</v>
+      </c>
+      <c r="X11" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="Y11" s="5">
         <v>1920</v>
       </c>
-      <c r="Y11" s="4">
+      <c r="Z11" s="4">
         <v>632800</v>
       </c>
-      <c r="Z11" s="5">
+      <c r="AA11" s="5">
         <v>22868427778</v>
       </c>
-      <c r="AA11" s="5">
+      <c r="AB11" s="5">
         <v>79665769974</v>
       </c>
-      <c r="AB11" s="2" t="s">
-        <v>74</v>
-      </c>
       <c r="AC11" s="2" t="s">
         <v>74</v>
       </c>
@@ -3143,10 +3287,10 @@
       <c r="AF11" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="AG11" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="AH11" s="5" t="s">
+      <c r="AG11" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="AH11" s="4" t="s">
         <v>74</v>
       </c>
       <c r="AI11" s="5" t="s">
@@ -3155,130 +3299,102 @@
       <c r="AJ11" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="AK11" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="AL11" s="5" t="s">
+      <c r="AK11" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="AL11" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="AM11" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="AM11" s="2">
+      <c r="AN11" s="2">
         <v>1</v>
       </c>
-      <c r="AN11" s="2">
+      <c r="AO11" s="2">
         <v>12</v>
       </c>
-      <c r="AO11" s="2">
+      <c r="AP11" s="2">
         <v>3</v>
       </c>
-      <c r="AP11" s="13">
+      <c r="AQ11" s="2">
         <v>3</v>
       </c>
-      <c r="AQ11" s="9">
+      <c r="AR11" s="7">
         <v>73</v>
       </c>
-      <c r="AR11" s="2" t="s">
+      <c r="AS11" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="AS11" s="2" t="s">
-        <v>70</v>
-      </c>
       <c r="AT11" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="AU11" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="AU11" s="2" t="s">
+      <c r="AV11" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="AV11" s="2" t="s">
-        <v>74</v>
-      </c>
       <c r="AW11" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="AX11" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="AX11" s="9">
+      <c r="AY11" s="7">
         <v>4708515</v>
       </c>
-      <c r="AY11" s="2">
+      <c r="AZ11" s="10">
         <v>30</v>
       </c>
-      <c r="AZ11" s="2">
-        <v>2007</v>
-      </c>
-      <c r="BA11" s="2">
+      <c r="BA11" s="13" t="s">
+        <v>193</v>
+      </c>
+      <c r="BB11" s="11">
         <v>9</v>
       </c>
-      <c r="BB11" s="2">
+      <c r="BC11" s="2">
         <v>5</v>
       </c>
-      <c r="BC11" s="2" t="s">
-        <v>69</v>
-      </c>
       <c r="BD11" s="2" t="s">
         <v>69</v>
       </c>
       <c r="BE11" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="BF11" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="BF11" s="2" t="s">
+      <c r="BG11" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="BG11" s="2" t="s">
+      <c r="BH11" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="BH11" s="13">
+      <c r="BI11" s="2">
         <v>16</v>
       </c>
-      <c r="BI11" s="9" t="s">
+      <c r="BJ11" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="BJ11" s="2">
+      <c r="BK11" s="2">
         <v>0.69</v>
       </c>
-      <c r="BK11" s="2" t="s">
+      <c r="BL11" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="BL11" s="2" t="s">
-        <v>69</v>
-      </c>
       <c r="BM11" s="2" t="s">
         <v>69</v>
       </c>
+      <c r="BN11" s="2" t="s">
+        <v>69</v>
+      </c>
     </row>
-    <row r="17" spans="61:63" x14ac:dyDescent="0.2">
-      <c r="BI17" s="14"/>
-      <c r="BJ17" s="15"/>
-      <c r="BK17" s="15"/>
-    </row>
-    <row r="18" spans="61:63" x14ac:dyDescent="0.2">
-      <c r="BI18" s="15"/>
-      <c r="BJ18" s="15"/>
-      <c r="BK18" s="15"/>
-    </row>
-    <row r="19" spans="61:63" x14ac:dyDescent="0.2">
-      <c r="BI19" s="15"/>
-      <c r="BJ19" s="15"/>
-      <c r="BK19" s="15"/>
-    </row>
-    <row r="20" spans="61:63" x14ac:dyDescent="0.2">
-      <c r="BI20" s="15"/>
-      <c r="BJ20" s="15"/>
-      <c r="BK20" s="15"/>
-    </row>
-    <row r="21" spans="61:63" x14ac:dyDescent="0.2">
-      <c r="BI21" s="15"/>
-      <c r="BJ21" s="15"/>
-      <c r="BK21" s="15"/>
-    </row>
-    <row r="22" spans="61:63" x14ac:dyDescent="0.2">
-      <c r="BI22" s="15"/>
-      <c r="BJ22" s="15"/>
-      <c r="BK22" s="15"/>
-    </row>
-    <row r="23" spans="61:63" x14ac:dyDescent="0.2">
-      <c r="BI23" s="15"/>
-      <c r="BJ23" s="15"/>
-      <c r="BK23" s="15"/>
+    <row r="17" spans="61:61">
+      <c r="BI17" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
vault backup: 2026-10-25 23:41:41
</commit_message>
<xml_diff>
--- a/Курс 3/Проектирование БД/Курисовая/Книга1.xlsx
+++ b/Курс 3/Проектирование БД/Курисовая/Книга1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11020"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OleSTEEP\Documents\Курисовая\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/olesteep/Documents/Study/Курс 3/Проектирование БД/Курисовая/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FCAEB80-577B-470E-AA03-8D5A2CB77EC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1384CB7A-F420-6940-BDE3-3B1536090A70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25695" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{E8ABD04A-C744-9645-AB57-F5C229AE1FFB}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{E8ABD04A-C744-9645-AB57-F5C229AE1FFB}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -663,7 +663,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -795,7 +795,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -817,9 +817,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1156,41 +1153,61 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66A0031D-02F4-BF44-AE14-59C0D6C26D55}">
   <dimension ref="A1:BN17"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.625" customWidth="1"/>
+    <col min="1" max="1" width="11.6640625" customWidth="1"/>
     <col min="5" max="5" width="13" customWidth="1"/>
-    <col min="6" max="6" width="12.125" customWidth="1"/>
+    <col min="6" max="6" width="12.1640625" customWidth="1"/>
     <col min="8" max="8" width="15.5" customWidth="1"/>
     <col min="9" max="9" width="12.5" customWidth="1"/>
-    <col min="10" max="10" width="12.875" customWidth="1"/>
-    <col min="13" max="13" width="12.125" customWidth="1"/>
-    <col min="15" max="15" width="28.625" bestFit="1" customWidth="1"/>
-    <col min="16" max="17" width="11" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="12.625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="15.625" customWidth="1"/>
-    <col min="20" max="20" width="14.75" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="22.375" customWidth="1"/>
-    <col min="26" max="26" width="15" customWidth="1"/>
-    <col min="27" max="27" width="14.375" customWidth="1"/>
-    <col min="28" max="28" width="25.5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.83203125" customWidth="1"/>
+    <col min="13" max="13" width="12.1640625" customWidth="1"/>
+    <col min="15" max="15" width="28.6640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="9.83203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="29.1640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="21.1640625" bestFit="1" customWidth="1"/>
+    <col min="23" max="24" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="25" max="26" width="9" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="14" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="26.1640625" bestFit="1" customWidth="1"/>
     <col min="31" max="31" width="11" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="14" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="14.625" customWidth="1"/>
-    <col min="38" max="38" width="21.125" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="13" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="13.875" customWidth="1"/>
-    <col min="47" max="47" width="12.875" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="23.875" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="13.125" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="21.625" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.875" customWidth="1"/>
-    <col min="61" max="61" width="17.125" customWidth="1"/>
-    <col min="62" max="62" width="12.125" customWidth="1"/>
-    <col min="63" max="63" width="13.125" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="11" bestFit="1" customWidth="1"/>
+    <col min="36" max="37" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="13.1640625" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="14.1640625" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="13" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="11.5" customWidth="1"/>
+    <col min="53" max="53" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="7.1640625" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="10" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="12" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="11.5" customWidth="1"/>
+    <col min="62" max="62" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="12" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="65" max="65" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="8.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:66" ht="63">
+    <row r="1" spans="1:66" ht="68" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1245,7 +1262,7 @@
       <c r="R1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="S1" s="14" t="s">
+      <c r="S1" s="1" t="s">
         <v>196</v>
       </c>
       <c r="T1" s="1" t="s">
@@ -1390,7 +1407,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="2" spans="1:66">
+    <row r="2" spans="1:66" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>177</v>
       </c>
@@ -1590,7 +1607,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="3" spans="1:66">
+    <row r="3" spans="1:66" ht="17" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>74</v>
       </c>
@@ -1790,7 +1807,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="4" spans="1:66">
+    <row r="4" spans="1:66" ht="17" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>173</v>
       </c>
@@ -1990,7 +2007,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="5" spans="1:66">
+    <row r="5" spans="1:66" ht="17" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>178</v>
       </c>
@@ -2190,7 +2207,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="6" spans="1:66">
+    <row r="6" spans="1:66" ht="17" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>74</v>
       </c>
@@ -2390,7 +2407,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="7" spans="1:66">
+    <row r="7" spans="1:66" ht="17" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>74</v>
       </c>
@@ -2590,7 +2607,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="8" spans="1:66">
+    <row r="8" spans="1:66" ht="17" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>74</v>
       </c>
@@ -2790,7 +2807,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="9" spans="1:66" ht="17.100000000000001" customHeight="1">
+    <row r="9" spans="1:66" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>169</v>
       </c>
@@ -2990,7 +3007,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="10" spans="1:66">
+    <row r="10" spans="1:66" ht="17" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>179</v>
       </c>
@@ -3190,7 +3207,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="11" spans="1:66">
+    <row r="11" spans="1:66" ht="17" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>74</v>
       </c>
@@ -3390,7 +3407,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="17" spans="61:61">
+    <row r="17" spans="61:61" x14ac:dyDescent="0.2">
       <c r="BI17" s="3"/>
     </row>
   </sheetData>

</xml_diff>